<commit_message>
docs: update (+ SQL breco schema)
</commit_message>
<xml_diff>
--- a/docs/tests/breco - Test Cases.xlsx
+++ b/docs/tests/breco - Test Cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp\www\breco_v2_0_0\docs\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FE090E6-5811-4441-A6E7-5FA10AACA449}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFB98999-FDF9-495D-AC44-64AF90DB878F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Story1 - Auth" sheetId="1" r:id="rId1"/>
@@ -25,15 +25,15 @@
     <sheet name="Story10 - Administer App" sheetId="10" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Story1 - Auth'!$A$3:$U$92</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Story2 - Pre-reg. Locations'!$A$3:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Story1 - Auth'!$A$3:$W$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Story2 - Pre-reg. Locations'!$A$3:$M$3</definedName>
   </definedNames>
   <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1208" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1424" uniqueCount="436">
   <si>
     <t>ID</t>
   </si>
@@ -1024,9 +1024,6 @@
     <t>Login flow + redirect</t>
   </si>
   <si>
-    <t>email = "toto@titi.com" &amp; password = "Toto1234" saisis en UI</t>
-  </si>
-  <si>
     <t>Display step 5 after successful registration</t>
   </si>
   <si>
@@ -1355,6 +1352,24 @@
   </si>
   <si>
     <t>Integration + Unit</t>
+  </si>
+  <si>
+    <t>Actual Result</t>
+  </si>
+  <si>
+    <t>Gap</t>
+  </si>
+  <si>
+    <t>As expected</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>email = "toto@titi.com" &amp; password = "Toto1234" entered in UI</t>
+  </si>
+  <si>
+    <t>To Implement</t>
   </si>
 </sst>
 </file>
@@ -1488,7 +1503,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1520,12 +1535,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC0C0C0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFC0C0C0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1597,13 +1623,7 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -1615,6 +1635,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1822,53 +1851,60 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U103"/>
+  <dimension ref="A1:W103"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="11.5703125" style="1"/>
-    <col min="3" max="3" width="20.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" style="1"/>
+    <col min="2" max="2" width="11.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" style="1" customWidth="1"/>
     <col min="5" max="5" width="25.85546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="15" style="1" customWidth="1"/>
-    <col min="7" max="7" width="38.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="34.42578125" style="1" customWidth="1"/>
     <col min="8" max="8" width="34.28515625" style="2" customWidth="1"/>
     <col min="9" max="9" width="43.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="28.140625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="17.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="11.5703125" style="1"/>
+    <col min="10" max="10" width="17.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="28.140625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="17.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="11.5703125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="26" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="L1" s="24"/>
+      <c r="M1" s="24"/>
+    </row>
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="23" t="s">
         <v>199</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
+      <c r="L2" s="24"/>
+      <c r="M2" s="24"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
@@ -1897,13 +1933,19 @@
         <v>204</v>
       </c>
       <c r="J3" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="K3" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="L3" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="9" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M3" s="9" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
         <v>5</v>
       </c>
@@ -1929,16 +1971,22 @@
         <v>9</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="J4" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L4" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="M4" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>10</v>
       </c>
@@ -1964,16 +2012,22 @@
         <v>11</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="J5" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L5" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K5" s="12" t="s">
+      <c r="M5" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
         <v>12</v>
       </c>
@@ -1999,16 +2053,22 @@
         <v>13</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="J6" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L6" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K6" s="12" t="s">
+      <c r="M6" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
         <v>14</v>
       </c>
@@ -2034,16 +2094,22 @@
         <v>15</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="J7" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L7" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="K7" s="13" t="s">
+      <c r="M7" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
         <v>16</v>
       </c>
@@ -2069,16 +2135,22 @@
         <v>17</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="J8" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L8" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K8" s="12" t="s">
+      <c r="M8" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
         <v>18</v>
       </c>
@@ -2104,16 +2176,22 @@
         <v>19</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="J9" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L9" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K9" s="12" t="s">
+      <c r="M9" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
         <v>20</v>
       </c>
@@ -2139,16 +2217,22 @@
         <v>22</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="J10" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K10" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L10" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K10" s="12" t="s">
+      <c r="M10" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
         <v>23</v>
       </c>
@@ -2174,16 +2258,22 @@
         <v>24</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="J11" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K11" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L11" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K11" s="13" t="s">
+      <c r="M11" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
         <v>25</v>
       </c>
@@ -2209,16 +2299,22 @@
         <v>26</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="J12" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K12" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L12" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K12" s="12" t="s">
+      <c r="M12" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
         <v>27</v>
       </c>
@@ -2244,16 +2340,22 @@
         <v>28</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="J13" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L13" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K13" s="12" t="s">
+      <c r="M13" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
         <v>29</v>
       </c>
@@ -2279,16 +2381,22 @@
         <v>30</v>
       </c>
       <c r="I14" s="15" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="J14" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K14" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L14" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K14" s="13" t="s">
+      <c r="M14" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
         <v>31</v>
       </c>
@@ -2314,16 +2422,22 @@
         <v>32</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="J15" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K15" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L15" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K15" s="12" t="s">
+      <c r="M15" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A16" s="21" t="s">
         <v>33</v>
       </c>
@@ -2349,16 +2463,22 @@
         <v>34</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="J16" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K16" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L16" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K16" s="12" t="s">
+      <c r="M16" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
         <v>35</v>
       </c>
@@ -2384,16 +2504,22 @@
         <v>36</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="J17" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K17" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L17" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K17" s="12" t="s">
+      <c r="M17" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="21" t="s">
         <v>37</v>
       </c>
@@ -2419,16 +2545,22 @@
         <v>38</v>
       </c>
       <c r="I18" s="15" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="J18" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K18" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L18" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K18" s="13" t="s">
+      <c r="M18" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A19" s="21" t="s">
         <v>39</v>
       </c>
@@ -2454,16 +2586,22 @@
         <v>40</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="J19" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K19" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L19" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K19" s="12" t="s">
+      <c r="M19" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A20" s="21" t="s">
         <v>41</v>
       </c>
@@ -2489,16 +2627,22 @@
         <v>42</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="J20" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K20" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L20" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K20" s="12" t="s">
+      <c r="M20" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
         <v>43</v>
       </c>
@@ -2524,16 +2668,22 @@
         <v>44</v>
       </c>
       <c r="I21" s="15" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="J21" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K21" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L21" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="K21" s="13" t="s">
+      <c r="M21" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A22" s="21" t="s">
         <v>45</v>
       </c>
@@ -2559,16 +2709,22 @@
         <v>46</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="J22" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K22" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L22" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K22" s="12" t="s">
+      <c r="M22" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="21" t="s">
         <v>47</v>
       </c>
@@ -2594,16 +2750,22 @@
         <v>48</v>
       </c>
       <c r="I23" s="15" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="J23" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K23" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L23" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K23" s="13" t="s">
+      <c r="M23" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="21" t="s">
         <v>49</v>
       </c>
@@ -2629,16 +2791,22 @@
         <v>50</v>
       </c>
       <c r="I24" s="15" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="J24" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K24" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L24" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K24" s="13" t="s">
+      <c r="M24" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="21" t="s">
         <v>51</v>
       </c>
@@ -2664,16 +2832,22 @@
         <v>52</v>
       </c>
       <c r="I25" s="15" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="J25" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K25" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L25" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K25" s="13" t="s">
+      <c r="M25" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="21" t="s">
         <v>53</v>
       </c>
@@ -2699,16 +2873,22 @@
         <v>54</v>
       </c>
       <c r="I26" s="15" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="J26" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K26" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L26" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K26" s="13" t="s">
+      <c r="M26" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A27" s="21" t="s">
         <v>55</v>
       </c>
@@ -2734,16 +2914,22 @@
         <v>56</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J27" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K27" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L27" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K27" s="12" t="s">
+      <c r="M27" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A28" s="21" t="s">
         <v>57</v>
       </c>
@@ -2769,16 +2955,22 @@
         <v>58</v>
       </c>
       <c r="I28" s="11" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J28" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K28" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L28" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K28" s="12" t="s">
+      <c r="M28" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="21" t="s">
         <v>59</v>
       </c>
@@ -2804,16 +2996,22 @@
         <v>60</v>
       </c>
       <c r="I29" s="17" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J29" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K29" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L29" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="K29" s="13" t="s">
+      <c r="M29" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A30" s="21" t="s">
         <v>61</v>
       </c>
@@ -2839,16 +3037,22 @@
         <v>62</v>
       </c>
       <c r="I30" s="11" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J30" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K30" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L30" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K30" s="12" t="s">
+      <c r="M30" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="21" t="s">
         <v>63</v>
       </c>
@@ -2874,16 +3078,22 @@
         <v>64</v>
       </c>
       <c r="I31" s="17" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J31" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K31" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L31" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K31" s="13" t="s">
+      <c r="M31" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="21" t="s">
         <v>65</v>
       </c>
@@ -2909,16 +3119,22 @@
         <v>66</v>
       </c>
       <c r="I32" s="17" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J32" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K32" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L32" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K32" s="13" t="s">
+      <c r="M32" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="21" t="s">
         <v>67</v>
       </c>
@@ -2944,16 +3160,22 @@
         <v>68</v>
       </c>
       <c r="I33" s="17" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J33" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K33" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L33" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K33" s="13" t="s">
+      <c r="M33" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="21" t="s">
         <v>69</v>
       </c>
@@ -2979,16 +3201,22 @@
         <v>70</v>
       </c>
       <c r="I34" s="17" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J34" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K34" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L34" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K34" s="13" t="s">
+      <c r="M34" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A35" s="21" t="s">
         <v>71</v>
       </c>
@@ -3014,16 +3242,22 @@
         <v>73</v>
       </c>
       <c r="I35" s="15" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="J35" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K35" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L35" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K35" s="12" t="s">
+      <c r="M35" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="21" t="s">
         <v>74</v>
       </c>
@@ -3049,16 +3283,22 @@
         <v>75</v>
       </c>
       <c r="I36" s="17" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J36" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K36" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L36" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K36" s="13" t="s">
+      <c r="M36" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="21" t="s">
         <v>76</v>
       </c>
@@ -3084,16 +3324,22 @@
         <v>77</v>
       </c>
       <c r="I37" s="17" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J37" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K37" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L37" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K37" s="13" t="s">
+      <c r="M37" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" s="21" t="s">
         <v>78</v>
       </c>
@@ -3119,16 +3365,22 @@
         <v>79</v>
       </c>
       <c r="I38" s="17" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="J38" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K38" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L38" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K38" s="12" t="s">
+      <c r="M38" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A39" s="21" t="s">
         <v>80</v>
       </c>
@@ -3148,22 +3400,28 @@
         <v>206</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="H39" s="16" t="s">
         <v>81</v>
       </c>
       <c r="I39" s="17" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J39" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K39" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L39" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K39" s="13" t="s">
+      <c r="M39" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" ht="15" x14ac:dyDescent="0.25">
       <c r="A40" s="21" t="s">
         <v>82</v>
       </c>
@@ -3189,16 +3447,22 @@
         <v>248</v>
       </c>
       <c r="I40" s="15" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="J40" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K40" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L40" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K40" s="12" t="s">
+      <c r="M40" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" ht="15" x14ac:dyDescent="0.25">
       <c r="A41" s="21" t="s">
         <v>83</v>
       </c>
@@ -3224,16 +3488,22 @@
         <v>250</v>
       </c>
       <c r="I41" s="15" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="J41" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K41" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L41" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K41" s="12" t="s">
+      <c r="M41" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" ht="15" x14ac:dyDescent="0.25">
       <c r="A42" s="21" t="s">
         <v>84</v>
       </c>
@@ -3259,16 +3529,22 @@
         <v>252</v>
       </c>
       <c r="I42" s="15" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="J42" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K42" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L42" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K42" s="12" t="s">
+      <c r="M42" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="21" t="s">
         <v>85</v>
       </c>
@@ -3294,16 +3570,22 @@
         <v>254</v>
       </c>
       <c r="I43" s="17" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="J43" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K43" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L43" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K43" s="13" t="s">
+      <c r="M43" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" ht="15" x14ac:dyDescent="0.25">
       <c r="A44" s="21" t="s">
         <v>86</v>
       </c>
@@ -3329,16 +3611,22 @@
         <v>256</v>
       </c>
       <c r="I44" s="17" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="J44" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K44" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L44" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="K44" s="13" t="s">
+      <c r="M44" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" ht="15" x14ac:dyDescent="0.25">
       <c r="A45" s="21" t="s">
         <v>87</v>
       </c>
@@ -3364,16 +3652,22 @@
         <v>258</v>
       </c>
       <c r="I45" s="15" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="J45" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K45" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L45" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K45" s="13" t="s">
+      <c r="M45" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" ht="15" x14ac:dyDescent="0.25">
       <c r="A46" s="21" t="s">
         <v>88</v>
       </c>
@@ -3399,16 +3693,22 @@
         <v>260</v>
       </c>
       <c r="I46" s="15" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="J46" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K46" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L46" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K46" s="13" t="s">
+      <c r="M46" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A47" s="21" t="s">
         <v>89</v>
       </c>
@@ -3434,16 +3734,22 @@
         <v>262</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="J47" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K47" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L47" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K47" s="12" t="s">
+      <c r="M47" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A48" s="21" t="s">
         <v>90</v>
       </c>
@@ -3469,16 +3775,22 @@
         <v>91</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="J48" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K48" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L48" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K48" s="12" t="s">
+      <c r="M48" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="49" spans="1:21" ht="15" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A49" s="21" t="s">
         <v>92</v>
       </c>
@@ -3504,16 +3816,22 @@
         <v>265</v>
       </c>
       <c r="I49" s="17" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="J49" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K49" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L49" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K49" s="13" t="s">
+      <c r="M49" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="50" spans="1:21" ht="15" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A50" s="21" t="s">
         <v>93</v>
       </c>
@@ -3539,16 +3857,22 @@
         <v>267</v>
       </c>
       <c r="I50" s="15" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="J50" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K50" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L50" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K50" s="13" t="s">
+      <c r="M50" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="51" spans="1:21" ht="15" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A51" s="21" t="s">
         <v>94</v>
       </c>
@@ -3574,16 +3898,22 @@
         <v>269</v>
       </c>
       <c r="I51" s="17" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="J51" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K51" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L51" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K51" s="13" t="s">
+      <c r="M51" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="52" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:23" ht="45" x14ac:dyDescent="0.25">
       <c r="A52" s="21" t="s">
         <v>95</v>
       </c>
@@ -3609,16 +3939,22 @@
         <v>271</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="J52" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K52" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L52" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K52" s="12" t="s">
+      <c r="M52" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="53" spans="1:21" ht="15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A53" s="21" t="s">
         <v>96</v>
       </c>
@@ -3644,16 +3980,22 @@
         <v>273</v>
       </c>
       <c r="I53" s="17" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="J53" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K53" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L53" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K53" s="13" t="s">
+      <c r="M53" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="54" spans="1:21" ht="15" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A54" s="21" t="s">
         <v>97</v>
       </c>
@@ -3679,16 +4021,22 @@
         <v>275</v>
       </c>
       <c r="I54" s="15" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="J54" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K54" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L54" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K54" s="13" t="s">
+      <c r="M54" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="55" spans="1:21" ht="15" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A55" s="21" t="s">
         <v>98</v>
       </c>
@@ -3714,16 +4062,22 @@
         <v>277</v>
       </c>
       <c r="I55" s="17" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J55" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K55" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L55" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K55" s="13" t="s">
+      <c r="M55" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="56" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:23" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="21" t="s">
         <v>99</v>
       </c>
@@ -3749,16 +4103,22 @@
         <v>279</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="J56" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K56" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L56" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K56" s="12" t="s">
+      <c r="M56" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="57" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="21" t="s">
         <v>100</v>
       </c>
@@ -3784,16 +4144,22 @@
         <v>281</v>
       </c>
       <c r="I57" s="17" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="J57" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K57" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L57" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K57" s="13" t="s">
+      <c r="M57" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="58" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="21" t="s">
         <v>101</v>
       </c>
@@ -3819,16 +4185,22 @@
         <v>283</v>
       </c>
       <c r="I58" s="15" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="J58" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K58" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L58" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K58" s="13" t="s">
+      <c r="M58" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="59" spans="1:21" ht="15" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A59" s="21" t="s">
         <v>102</v>
       </c>
@@ -3854,16 +4226,22 @@
         <v>285</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="J59" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K59" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L59" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K59" s="12" t="s">
+      <c r="M59" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="60" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:23" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A60" s="21" t="s">
         <v>103</v>
       </c>
@@ -3889,16 +4267,22 @@
         <v>287</v>
       </c>
       <c r="I60" s="11" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="J60" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K60" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L60" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K60" s="12" t="s">
+      <c r="M60" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="61" spans="1:21" ht="15" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A61" s="21" t="s">
         <v>104</v>
       </c>
@@ -3924,16 +4308,22 @@
         <v>289</v>
       </c>
       <c r="I61" s="17" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J61" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K61" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L61" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="K61" s="13" t="s">
+      <c r="M61" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="62" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:23" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A62" s="21" t="s">
         <v>123</v>
       </c>
@@ -3956,19 +4346,25 @@
         <v>301</v>
       </c>
       <c r="H62" s="11" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="J62" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K62" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L62" s="11" t="s">
         <v>296</v>
       </c>
-      <c r="K62" s="13" t="s">
+      <c r="M62" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="63" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:23" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A63" s="21" t="s">
         <v>127</v>
       </c>
@@ -3991,19 +4387,25 @@
         <v>302</v>
       </c>
       <c r="H63" s="11" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="J63" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K63" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L63" s="11" t="s">
         <v>296</v>
       </c>
-      <c r="K63" s="12" t="s">
+      <c r="M63" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="64" spans="1:21" s="7" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:23" s="7" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A64" s="21" t="s">
         <v>128</v>
       </c>
@@ -4029,16 +4431,20 @@
         <v>130</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="J64" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K64" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L64" s="11" t="s">
         <v>296</v>
       </c>
-      <c r="K64" s="12" t="s">
+      <c r="M64" s="12" t="s">
         <v>209</v>
       </c>
-      <c r="L64" s="1"/>
-      <c r="M64" s="1"/>
       <c r="N64" s="1"/>
       <c r="O64" s="1"/>
       <c r="P64" s="1"/>
@@ -4047,8 +4453,10 @@
       <c r="S64" s="1"/>
       <c r="T64" s="1"/>
       <c r="U64" s="1"/>
-    </row>
-    <row r="65" spans="1:21" s="7" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="V64" s="1"/>
+      <c r="W64" s="1"/>
+    </row>
+    <row r="65" spans="1:23" s="7" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A65" s="21" t="s">
         <v>133</v>
       </c>
@@ -4071,19 +4479,23 @@
         <v>306</v>
       </c>
       <c r="H65" s="11" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="J65" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K65" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L65" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K65" s="12" t="s">
+      <c r="M65" s="12" t="s">
         <v>209</v>
       </c>
-      <c r="L65" s="1"/>
-      <c r="M65" s="1"/>
       <c r="N65" s="1"/>
       <c r="O65" s="1"/>
       <c r="P65" s="1"/>
@@ -4092,8 +4504,10 @@
       <c r="S65" s="1"/>
       <c r="T65" s="1"/>
       <c r="U65" s="1"/>
-    </row>
-    <row r="66" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="V65" s="1"/>
+      <c r="W65" s="1"/>
+    </row>
+    <row r="66" spans="1:23" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A66" s="21" t="s">
         <v>134</v>
       </c>
@@ -4116,19 +4530,25 @@
         <v>307</v>
       </c>
       <c r="H66" s="11" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J66" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K66" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L66" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K66" s="12" t="s">
+      <c r="M66" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="67" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:23" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A67" s="21" t="s">
         <v>135</v>
       </c>
@@ -4151,19 +4571,25 @@
         <v>308</v>
       </c>
       <c r="H67" s="11" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="I67" s="11" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="J67" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K67" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L67" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K67" s="12" t="s">
+      <c r="M67" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="68" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:23" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A68" s="21" t="s">
         <v>154</v>
       </c>
@@ -4183,22 +4609,28 @@
         <v>206</v>
       </c>
       <c r="G68" s="11" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H68" s="11" t="s">
         <v>155</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="J68" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K68" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L68" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K68" s="12" t="s">
+      <c r="M68" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="69" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:23" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A69" s="21" t="s">
         <v>156</v>
       </c>
@@ -4218,22 +4650,28 @@
         <v>206</v>
       </c>
       <c r="G69" s="11" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H69" s="11" t="s">
         <v>157</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="J69" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K69" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L69" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K69" s="12" t="s">
+      <c r="M69" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="70" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:23" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A70" s="21" t="s">
         <v>161</v>
       </c>
@@ -4253,22 +4691,28 @@
         <v>294</v>
       </c>
       <c r="G70" s="11" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="H70" s="11" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="J70" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K70" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L70" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K70" s="12" t="s">
+      <c r="M70" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="71" spans="1:21" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:23" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A71" s="11" t="s">
         <v>166</v>
       </c>
@@ -4288,27 +4732,33 @@
         <v>294</v>
       </c>
       <c r="G71" s="11" t="s">
+        <v>328</v>
+      </c>
+      <c r="H71" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="I71" s="11" t="s">
+        <v>381</v>
+      </c>
+      <c r="J71" s="11" t="s">
+        <v>435</v>
+      </c>
+      <c r="K71" s="11" t="s">
+        <v>435</v>
+      </c>
+      <c r="L71" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="M71" s="20" t="s">
         <v>329</v>
       </c>
-      <c r="H71" s="11" t="s">
-        <v>427</v>
-      </c>
-      <c r="I71" s="11" t="s">
-        <v>382</v>
-      </c>
-      <c r="J71" s="11" t="s">
-        <v>211</v>
-      </c>
-      <c r="K71" s="20" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="72" spans="1:21" ht="38.25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="72" spans="1:23" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A72" s="21" t="s">
         <v>105</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C72" s="11" t="s">
         <v>106</v>
@@ -4332,18 +4782,24 @@
         <v>110</v>
       </c>
       <c r="J72" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K72" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L72" s="11" t="s">
         <v>292</v>
       </c>
-      <c r="K72" s="13" t="s">
+      <c r="M72" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="73" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:23" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A73" s="21" t="s">
         <v>111</v>
       </c>
       <c r="B73" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C73" s="11" t="s">
         <v>106</v>
@@ -4361,24 +4817,30 @@
         <v>293</v>
       </c>
       <c r="H73" s="11" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="I73" s="11" t="s">
         <v>112</v>
       </c>
       <c r="J73" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K73" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L73" s="11" t="s">
         <v>292</v>
       </c>
-      <c r="K73" s="12" t="s">
+      <c r="M73" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="74" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:23" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A74" s="21" t="s">
         <v>113</v>
       </c>
       <c r="B74" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C74" s="11" t="s">
         <v>106</v>
@@ -4399,16 +4861,22 @@
         <v>115</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="J74" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K74" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L74" s="11" t="s">
         <v>296</v>
       </c>
-      <c r="K74" s="12" t="s">
+      <c r="M74" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="75" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:23" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A75" s="21" t="s">
         <v>136</v>
       </c>
@@ -4434,16 +4902,22 @@
         <v>140</v>
       </c>
       <c r="I75" s="11" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="J75" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K75" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L75" s="11" t="s">
         <v>296</v>
       </c>
-      <c r="K75" s="13" t="s">
+      <c r="M75" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="76" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:23" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A76" s="21" t="s">
         <v>141</v>
       </c>
@@ -4469,16 +4943,22 @@
         <v>311</v>
       </c>
       <c r="I76" s="11" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="J76" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K76" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L76" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K76" s="12" t="s">
+      <c r="M76" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="77" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:23" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A77" s="21" t="s">
         <v>142</v>
       </c>
@@ -4504,16 +4984,22 @@
         <v>313</v>
       </c>
       <c r="I77" s="11" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="J77" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K77" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L77" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K77" s="12" t="s">
+      <c r="M77" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="78" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:23" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A78" s="21" t="s">
         <v>143</v>
       </c>
@@ -4539,16 +5025,22 @@
         <v>315</v>
       </c>
       <c r="I78" s="11" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="J78" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K78" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L78" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K78" s="13" t="s">
+      <c r="M78" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="79" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:23" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A79" s="21" t="s">
         <v>144</v>
       </c>
@@ -4577,13 +5069,19 @@
         <v>145</v>
       </c>
       <c r="J79" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K79" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L79" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K79" s="12" t="s">
+      <c r="M79" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="80" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:23" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A80" s="21" t="s">
         <v>146</v>
       </c>
@@ -4609,16 +5107,22 @@
         <v>318</v>
       </c>
       <c r="I80" s="11" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="J80" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K80" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L80" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K80" s="13" t="s">
+      <c r="M80" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A81" s="21" t="s">
         <v>150</v>
       </c>
@@ -4641,19 +5145,25 @@
         <v>319</v>
       </c>
       <c r="H81" s="11" t="s">
-        <v>320</v>
+        <v>434</v>
       </c>
       <c r="I81" s="11" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="J81" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K81" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L81" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K81" s="13" t="s">
+      <c r="M81" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A82" s="21" t="s">
         <v>152</v>
       </c>
@@ -4673,27 +5183,33 @@
         <v>206</v>
       </c>
       <c r="G82" s="11" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H82" s="11" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="I82" s="11" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J82" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K82" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L82" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K82" s="13" t="s">
+      <c r="M82" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="83" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A83" s="21" t="s">
         <v>116</v>
       </c>
       <c r="B83" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C83" s="11" t="s">
         <v>106</v>
@@ -4714,21 +5230,27 @@
         <v>30</v>
       </c>
       <c r="I83" s="11" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="J83" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K83" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L83" s="11" t="s">
         <v>292</v>
       </c>
-      <c r="K83" s="13" t="s">
+      <c r="M83" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="84" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A84" s="21" t="s">
         <v>117</v>
       </c>
       <c r="B84" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C84" s="11" t="s">
         <v>106</v>
@@ -4749,16 +5271,22 @@
         <v>118</v>
       </c>
       <c r="I84" s="11" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="J84" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K84" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L84" s="11" t="s">
         <v>296</v>
       </c>
-      <c r="K84" s="12" t="s">
+      <c r="M84" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="85" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A85" s="21" t="s">
         <v>158</v>
       </c>
@@ -4775,30 +5303,36 @@
         <v>159</v>
       </c>
       <c r="F85" s="11" t="s">
+        <v>323</v>
+      </c>
+      <c r="G85" s="11" t="s">
         <v>324</v>
       </c>
-      <c r="G85" s="11" t="s">
-        <v>325</v>
-      </c>
       <c r="H85" s="11" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="I85" s="11" t="s">
         <v>160</v>
       </c>
       <c r="J85" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K85" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L85" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K85" s="13" t="s">
+      <c r="M85" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="86" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A86" s="21" t="s">
         <v>119</v>
       </c>
       <c r="B86" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C86" s="11" t="s">
         <v>106</v>
@@ -4822,13 +5356,19 @@
         <v>122</v>
       </c>
       <c r="J86" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K86" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L86" s="11" t="s">
         <v>292</v>
       </c>
-      <c r="K86" s="13" t="s">
+      <c r="M86" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A87" s="21" t="s">
         <v>162</v>
       </c>
@@ -4848,22 +5388,28 @@
         <v>206</v>
       </c>
       <c r="G87" s="11" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="H87" s="11" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="I87" s="11" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="J87" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K87" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L87" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K87" s="12" t="s">
+      <c r="M87" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="88" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="21" t="s">
         <v>164</v>
       </c>
@@ -4883,27 +5429,33 @@
         <v>294</v>
       </c>
       <c r="G88" s="11" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="H88" s="11" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="I88" s="11" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="J88" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K88" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L88" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K88" s="12" t="s">
+      <c r="M88" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="89" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A89" s="21" t="s">
         <v>131</v>
       </c>
       <c r="B89" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C89" s="11" t="s">
         <v>106</v>
@@ -4924,16 +5476,22 @@
         <v>132</v>
       </c>
       <c r="I89" s="11" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="J89" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K89" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L89" s="11" t="s">
         <v>296</v>
       </c>
-      <c r="K89" s="12" t="s">
+      <c r="M89" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A90" s="21" t="s">
         <v>168</v>
       </c>
@@ -4953,22 +5511,28 @@
         <v>294</v>
       </c>
       <c r="G90" s="11" t="s">
+        <v>330</v>
+      </c>
+      <c r="H90" s="11" t="s">
         <v>331</v>
       </c>
-      <c r="H90" s="11" t="s">
-        <v>332</v>
-      </c>
       <c r="I90" s="11" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="J90" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K90" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L90" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K90" s="12" t="s">
+      <c r="M90" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="91" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A91" s="21" t="s">
         <v>170</v>
       </c>
@@ -4988,22 +5552,28 @@
         <v>294</v>
       </c>
       <c r="G91" s="11" t="s">
+        <v>332</v>
+      </c>
+      <c r="H91" s="11" t="s">
         <v>333</v>
       </c>
-      <c r="H91" s="11" t="s">
-        <v>334</v>
-      </c>
       <c r="I91" s="11" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="J91" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K91" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L91" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K91" s="13" t="s">
+      <c r="M91" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="92" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A92" s="21" t="s">
         <v>171</v>
       </c>
@@ -5023,22 +5593,28 @@
         <v>294</v>
       </c>
       <c r="G92" s="15" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="H92" s="16" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="I92" s="11" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="J92" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K92" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L92" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="K92" s="12" t="s">
+      <c r="M92" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="93" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="5"/>
       <c r="B93" s="5"/>
       <c r="C93" s="5"/>
@@ -5050,8 +5626,10 @@
       <c r="I93" s="5"/>
       <c r="J93" s="5"/>
       <c r="K93" s="5"/>
-    </row>
-    <row r="94" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L93" s="5"/>
+      <c r="M93" s="5"/>
+    </row>
+    <row r="94" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="5"/>
       <c r="B94" s="5"/>
       <c r="C94" s="5"/>
@@ -5063,8 +5641,10 @@
       <c r="I94" s="5"/>
       <c r="J94" s="5"/>
       <c r="K94" s="5"/>
-    </row>
-    <row r="95" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L94" s="5"/>
+      <c r="M94" s="5"/>
+    </row>
+    <row r="95" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="5"/>
       <c r="B95" s="5"/>
       <c r="C95" s="5"/>
@@ -5076,8 +5656,10 @@
       <c r="I95" s="5"/>
       <c r="J95" s="5"/>
       <c r="K95" s="5"/>
-    </row>
-    <row r="96" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L95" s="5"/>
+      <c r="M95" s="5"/>
+    </row>
+    <row r="96" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="5"/>
       <c r="B96" s="5"/>
       <c r="C96" s="5"/>
@@ -5089,8 +5671,10 @@
       <c r="I96" s="5"/>
       <c r="J96" s="5"/>
       <c r="K96" s="5"/>
-    </row>
-    <row r="97" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L96" s="5"/>
+      <c r="M96" s="5"/>
+    </row>
+    <row r="97" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="5"/>
       <c r="B97" s="5"/>
       <c r="C97" s="5"/>
@@ -5102,8 +5686,10 @@
       <c r="I97" s="5"/>
       <c r="J97" s="5"/>
       <c r="K97" s="5"/>
-    </row>
-    <row r="98" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L97" s="5"/>
+      <c r="M97" s="5"/>
+    </row>
+    <row r="98" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="5"/>
       <c r="B98" s="5"/>
       <c r="C98" s="5"/>
@@ -5115,8 +5701,10 @@
       <c r="I98" s="5"/>
       <c r="J98" s="5"/>
       <c r="K98" s="5"/>
-    </row>
-    <row r="99" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L98" s="5"/>
+      <c r="M98" s="5"/>
+    </row>
+    <row r="99" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="5"/>
       <c r="B99" s="5"/>
       <c r="C99" s="5"/>
@@ -5128,8 +5716,10 @@
       <c r="I99" s="5"/>
       <c r="J99" s="5"/>
       <c r="K99" s="5"/>
-    </row>
-    <row r="100" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L99" s="5"/>
+      <c r="M99" s="5"/>
+    </row>
+    <row r="100" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="5"/>
       <c r="B100" s="5"/>
       <c r="C100" s="5"/>
@@ -5141,8 +5731,10 @@
       <c r="I100" s="5"/>
       <c r="J100" s="5"/>
       <c r="K100" s="5"/>
-    </row>
-    <row r="101" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L100" s="5"/>
+      <c r="M100" s="5"/>
+    </row>
+    <row r="101" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="5"/>
       <c r="B101" s="5"/>
       <c r="C101" s="5"/>
@@ -5154,8 +5746,10 @@
       <c r="I101" s="5"/>
       <c r="J101" s="5"/>
       <c r="K101" s="5"/>
-    </row>
-    <row r="102" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L101" s="5"/>
+      <c r="M101" s="5"/>
+    </row>
+    <row r="102" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="5"/>
       <c r="B102" s="5"/>
       <c r="C102" s="5"/>
@@ -5167,8 +5761,10 @@
       <c r="I102" s="5"/>
       <c r="J102" s="5"/>
       <c r="K102" s="5"/>
-    </row>
-    <row r="103" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L102" s="5"/>
+      <c r="M102" s="5"/>
+    </row>
+    <row r="103" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="5"/>
       <c r="B103" s="5"/>
       <c r="C103" s="5"/>
@@ -5180,16 +5776,18 @@
       <c r="I103" s="5"/>
       <c r="J103" s="5"/>
       <c r="K103" s="5"/>
+      <c r="L103" s="5"/>
+      <c r="M103" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:U92" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A62:U89">
+  <autoFilter ref="A3:W92" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A62:W89">
       <sortCondition ref="C3:C92"/>
     </sortState>
   </autoFilter>
   <mergeCells count="2">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation operator="equal" sqref="H1:H39 H64:H1067" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -5208,36 +5806,36 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="29" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
-        <v>347</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-    </row>
-    <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+    </row>
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="31" t="s">
+        <v>346</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+    </row>
+    <row r="3" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -5265,11 +5863,17 @@
       <c r="I3" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="K3" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>429</v>
+      <c r="M3" s="3" t="s">
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -5294,50 +5898,56 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="11.5703125" style="8"/>
     <col min="5" max="5" width="25" style="8" customWidth="1"/>
     <col min="6" max="6" width="21.7109375" style="8" customWidth="1"/>
     <col min="7" max="7" width="44" style="8" customWidth="1"/>
-    <col min="8" max="8" width="48.28515625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="23.5703125" style="8" customWidth="1"/>
     <col min="9" max="9" width="38.42578125" style="8" customWidth="1"/>
-    <col min="10" max="10" width="13.28515625" style="8" customWidth="1"/>
-    <col min="11" max="16384" width="11.5703125" style="8"/>
+    <col min="10" max="10" width="16.28515625" style="8" customWidth="1"/>
+    <col min="11" max="11" width="9.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.28515625" style="8" customWidth="1"/>
+    <col min="13" max="16384" width="11.5703125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:13" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="26" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-    </row>
-    <row r="2" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
-        <v>336</v>
-      </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-    </row>
-    <row r="3" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+    </row>
+    <row r="2" spans="1:13" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
+        <v>335</v>
+      </c>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
+      <c r="L2" s="28"/>
+      <c r="M2" s="28"/>
+    </row>
+    <row r="3" spans="1:13" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
@@ -5366,13 +5976,19 @@
         <v>204</v>
       </c>
       <c r="J3" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="K3" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="L3" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="9" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M3" s="9" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
         <v>173</v>
       </c>
@@ -5389,25 +6005,31 @@
         <v>174</v>
       </c>
       <c r="F4" s="11" t="s">
+        <v>336</v>
+      </c>
+      <c r="G4" s="11" t="s">
         <v>337</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>338</v>
       </c>
       <c r="H4" s="11" t="s">
         <v>175</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="J4" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L4" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="M4" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>176</v>
       </c>
@@ -5424,25 +6046,31 @@
         <v>174</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>177</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="J5" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L5" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K5" s="12" t="s">
+      <c r="M5" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
         <v>178</v>
       </c>
@@ -5459,30 +6087,36 @@
         <v>174</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="H6" s="11" t="s">
         <v>179</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>341</v>
-      </c>
-      <c r="K6" s="12" t="s">
+        <v>432</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L6" s="11" t="s">
+        <v>340</v>
+      </c>
+      <c r="M6" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="51" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="51" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
         <v>180</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>106</v>
@@ -5494,30 +6128,36 @@
         <v>181</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="H7" s="11" t="s">
         <v>182</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="J7" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L7" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="K7" s="12" t="s">
+      <c r="M7" s="12" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="165.75" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
         <v>183</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>106</v>
@@ -5529,10 +6169,10 @@
         <v>181</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="H8" s="11" t="s">
         <v>184</v>
@@ -5541,18 +6181,24 @@
         <v>185</v>
       </c>
       <c r="J8" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L8" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="K8" s="13" t="s">
+      <c r="M8" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="127.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" ht="127.5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
         <v>186</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>106</v>
@@ -5564,10 +6210,10 @@
         <v>181</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="H9" s="11" t="s">
         <v>187</v>
@@ -5576,18 +6222,24 @@
         <v>188</v>
       </c>
       <c r="J9" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L9" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="K9" s="13" t="s">
+      <c r="M9" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
         <v>189</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>106</v>
@@ -5599,10 +6251,10 @@
         <v>181</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="H10" s="11" t="s">
         <v>190</v>
@@ -5611,18 +6263,24 @@
         <v>191</v>
       </c>
       <c r="J10" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K10" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L10" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="K10" s="13" t="s">
+      <c r="M10" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="165.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="165.75" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
         <v>192</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>106</v>
@@ -5634,10 +6292,10 @@
         <v>181</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="H11" s="11" t="s">
         <v>193</v>
@@ -5646,13 +6304,19 @@
         <v>194</v>
       </c>
       <c r="J11" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K11" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L11" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="K11" s="13" t="s">
+      <c r="M11" s="13" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
         <v>195</v>
       </c>
@@ -5669,29 +6333,35 @@
         <v>196</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="H12" s="11" t="s">
         <v>197</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="J12" s="11" t="s">
-        <v>341</v>
-      </c>
-      <c r="K12" s="12" t="s">
+        <v>432</v>
+      </c>
+      <c r="K12" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="L12" s="11" t="s">
+        <v>340</v>
+      </c>
+      <c r="M12" s="12" t="s">
         <v>209</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:K3" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A3:M3" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation operator="equal" sqref="H1:H3" xr:uid="{00000000-0002-0000-0100-000000000000}">
@@ -5714,39 +6384,43 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="29" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
-        <v>354</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-    </row>
-    <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+    </row>
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="31" t="s">
+        <v>353</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+    </row>
+    <row r="3" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -5774,17 +6448,23 @@
       <c r="I3" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="K3" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>429</v>
+      <c r="M3" s="3" t="s">
+        <v>428</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:L2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation operator="equal" sqref="G2 H1 H3" xr:uid="{42C6FC0F-3EAA-4656-AAA7-DA666910C92F}">
@@ -5803,36 +6483,36 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="29" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
-        <v>353</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-    </row>
-    <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+    </row>
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="31" t="s">
+        <v>352</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+    </row>
+    <row r="3" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -5860,11 +6540,17 @@
       <c r="I3" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="K3" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>429</v>
+      <c r="M3" s="3" t="s">
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -5889,36 +6575,36 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="29" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
-        <v>352</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-    </row>
-    <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+    </row>
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="31" t="s">
+        <v>351</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+    </row>
+    <row r="3" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -5946,11 +6632,17 @@
       <c r="I3" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="K3" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>429</v>
+      <c r="M3" s="3" t="s">
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -5975,36 +6667,36 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="29" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
-        <v>351</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-    </row>
-    <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+    </row>
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="31" t="s">
+        <v>350</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+    </row>
+    <row r="3" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -6032,11 +6724,17 @@
       <c r="I3" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="K3" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>429</v>
+      <c r="M3" s="3" t="s">
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -6061,36 +6759,36 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="29" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
-        <v>350</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-    </row>
-    <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+    </row>
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="31" t="s">
+        <v>349</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+    </row>
+    <row r="3" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -6118,11 +6816,17 @@
       <c r="I3" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="K3" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>429</v>
+      <c r="M3" s="3" t="s">
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -6147,36 +6851,36 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="29" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="31" t="s">
-        <v>349</v>
-      </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-    </row>
-    <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+    </row>
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="32" t="s">
+        <v>348</v>
+      </c>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+    </row>
+    <row r="3" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -6204,11 +6908,17 @@
       <c r="I3" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="K3" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>429</v>
+      <c r="M3" s="3" t="s">
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -6233,36 +6943,36 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="29" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
-        <v>348</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-    </row>
-    <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+    </row>
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="31" t="s">
+        <v>347</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+    </row>
+    <row r="3" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -6290,11 +7000,17 @@
       <c r="I3" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="K3" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>429</v>
+      <c r="M3" s="3" t="s">
+        <v>428</v>
       </c>
     </row>
   </sheetData>

</xml_diff>